<commit_message>
Upload Y4_B2526_General_&_Special_Internal_1_A1_reference_data.xlsx via attendance app
</commit_message>
<xml_diff>
--- a/reference_data/Y4_B2526_General_&_Special_Internal_1_A1_reference_data.xlsx
+++ b/reference_data/Y4_B2526_General_&_Special_Internal_1_A1_reference_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\moham\Desktop\reference_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dr_ma\Desktop\reference_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BAFD4FC-8E77-405B-AEDC-B470DFB40314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F0C2A14-E797-4BA3-A459-875A2D0254C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2900" yWindow="370" windowWidth="18280" windowHeight="13100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2135" uniqueCount="863">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2171" uniqueCount="873">
   <si>
     <t>Student ID</t>
   </si>
@@ -2609,6 +2609,36 @@
   </si>
   <si>
     <t>unknown</t>
+  </si>
+  <si>
+    <t>Malony Ngong Deng Maathiei</t>
+  </si>
+  <si>
+    <t>ابراهيم عصفور ابراهيم رشوان عطا</t>
+  </si>
+  <si>
+    <t>عمار ياسر الصادق محمد</t>
+  </si>
+  <si>
+    <t>فادى عبد الله جميل شولى</t>
+  </si>
+  <si>
+    <t>طارق زياد محمود</t>
+  </si>
+  <si>
+    <t>مازن ايمن محمود عبدربه</t>
+  </si>
+  <si>
+    <t>يوسف محمد عبد المجيد مخلوف</t>
+  </si>
+  <si>
+    <t>جيوفانى جورج ميخائيل عطا الله</t>
+  </si>
+  <si>
+    <t>نور الهدى ياسر زين العابدين الحاج</t>
+  </si>
+  <si>
+    <t>ربا احمد محمد النجار</t>
   </si>
 </sst>
 </file>
@@ -2994,8 +3024,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E427"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:E438"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="46" customWidth="1"/>
@@ -3004,7 +3034,7 @@
     <col min="5" max="5" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3021,7 +3051,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>160</v>
       </c>
@@ -3038,7 +3068,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>315</v>
       </c>
@@ -3055,7 +3085,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
         <v>163</v>
       </c>
@@ -3072,7 +3102,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
         <v>679</v>
       </c>
@@ -3089,7 +3119,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
         <v>165</v>
       </c>
@@ -3106,7 +3136,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
         <v>167</v>
       </c>
@@ -3123,7 +3153,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">
         <v>169</v>
       </c>
@@ -3140,7 +3170,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
         <v>171</v>
       </c>
@@ -3157,7 +3187,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A10" s="2" t="s">
         <v>173</v>
       </c>
@@ -3174,7 +3204,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
         <v>175</v>
       </c>
@@ -3191,7 +3221,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
         <v>177</v>
       </c>
@@ -3208,7 +3238,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A13" s="3" t="s">
         <v>179</v>
       </c>
@@ -3225,7 +3255,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
         <v>181</v>
       </c>
@@ -3242,7 +3272,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A15" s="3" t="s">
         <v>183</v>
       </c>
@@ -3259,7 +3289,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A16" s="2" t="s">
         <v>185</v>
       </c>
@@ -3276,7 +3306,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" s="3" t="s">
         <v>187</v>
       </c>
@@ -3293,7 +3323,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A18" s="2" t="s">
         <v>189</v>
       </c>
@@ -3310,7 +3340,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A19" s="3" t="s">
         <v>191</v>
       </c>
@@ -3327,7 +3357,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A20" s="2" t="s">
         <v>193</v>
       </c>
@@ -3344,7 +3374,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A21" s="3" t="s">
         <v>195</v>
       </c>
@@ -3361,7 +3391,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A22" s="2" t="s">
         <v>682</v>
       </c>
@@ -3378,7 +3408,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A23" s="3" t="s">
         <v>684</v>
       </c>
@@ -3395,7 +3425,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A24" s="2" t="s">
         <v>197</v>
       </c>
@@ -3412,7 +3442,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A25" s="2" t="s">
         <v>686</v>
       </c>
@@ -3423,13 +3453,13 @@
         <v>7</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>681</v>
+        <v>500</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A26" s="3" t="s">
         <v>199</v>
       </c>
@@ -3446,7 +3476,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A27" s="2" t="s">
         <v>201</v>
       </c>
@@ -3463,12 +3493,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A28" s="2" t="s">
         <v>317</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>7</v>
@@ -3480,7 +3510,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A29" s="3" t="s">
         <v>203</v>
       </c>
@@ -3497,7 +3527,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A30" s="2" t="s">
         <v>205</v>
       </c>
@@ -3514,7 +3544,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A31" s="3" t="s">
         <v>207</v>
       </c>
@@ -3531,7 +3561,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
         <v>209</v>
       </c>
@@ -3548,7 +3578,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A33" s="3" t="s">
         <v>211</v>
       </c>
@@ -3565,7 +3595,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A34" s="2" t="s">
         <v>213</v>
       </c>
@@ -3582,7 +3612,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A35" s="3" t="s">
         <v>215</v>
       </c>
@@ -3599,7 +3629,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A36" s="2" t="s">
         <v>217</v>
       </c>
@@ -3616,7 +3646,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A37" s="3" t="s">
         <v>219</v>
       </c>
@@ -3633,7 +3663,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
         <v>221</v>
       </c>
@@ -3650,7 +3680,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A39" s="3" t="s">
         <v>223</v>
       </c>
@@ -3667,7 +3697,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A40" s="2" t="s">
         <v>225</v>
       </c>
@@ -3684,7 +3714,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A41" s="3" t="s">
         <v>227</v>
       </c>
@@ -3701,7 +3731,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A42" s="2" t="s">
         <v>229</v>
       </c>
@@ -3718,7 +3748,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A43" s="3" t="s">
         <v>231</v>
       </c>
@@ -3735,7 +3765,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A44" s="2" t="s">
         <v>233</v>
       </c>
@@ -3752,7 +3782,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A45" s="3" t="s">
         <v>235</v>
       </c>
@@ -3769,7 +3799,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A46" s="2" t="s">
         <v>237</v>
       </c>
@@ -3786,7 +3816,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A47" s="3" t="s">
         <v>239</v>
       </c>
@@ -3803,7 +3833,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A48" s="2" t="s">
         <v>241</v>
       </c>
@@ -3820,7 +3850,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A49" s="3" t="s">
         <v>243</v>
       </c>
@@ -3837,7 +3867,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A50" s="2" t="s">
         <v>245</v>
       </c>
@@ -3854,7 +3884,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A51" s="3" t="s">
         <v>247</v>
       </c>
@@ -3871,7 +3901,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A52" s="2" t="s">
         <v>249</v>
       </c>
@@ -3888,7 +3918,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A53" s="3" t="s">
         <v>251</v>
       </c>
@@ -3905,7 +3935,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A54" s="2" t="s">
         <v>253</v>
       </c>
@@ -3922,7 +3952,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A55" s="3" t="s">
         <v>255</v>
       </c>
@@ -3939,7 +3969,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A56" s="3" t="s">
         <v>318</v>
       </c>
@@ -3956,7 +3986,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A57" s="2" t="s">
         <v>320</v>
       </c>
@@ -3973,7 +4003,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A58" s="3" t="s">
         <v>322</v>
       </c>
@@ -3990,7 +4020,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A59" s="2" t="s">
         <v>324</v>
       </c>
@@ -4007,7 +4037,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A60" s="3" t="s">
         <v>326</v>
       </c>
@@ -4024,7 +4054,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A61" s="2" t="s">
         <v>328</v>
       </c>
@@ -4041,7 +4071,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A62" s="3" t="s">
         <v>330</v>
       </c>
@@ -4058,7 +4088,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A63" s="2" t="s">
         <v>332</v>
       </c>
@@ -4075,7 +4105,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A64" s="3" t="s">
         <v>334</v>
       </c>
@@ -4092,7 +4122,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A65" s="2" t="s">
         <v>336</v>
       </c>
@@ -4109,7 +4139,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A66" s="3" t="s">
         <v>338</v>
       </c>
@@ -4126,7 +4156,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A67" s="2" t="s">
         <v>340</v>
       </c>
@@ -4143,7 +4173,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A68" s="3" t="s">
         <v>342</v>
       </c>
@@ -4160,7 +4190,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A69" s="2" t="s">
         <v>344</v>
       </c>
@@ -4177,7 +4207,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A70" s="3" t="s">
         <v>346</v>
       </c>
@@ -4194,7 +4224,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A71" s="2" t="s">
         <v>348</v>
       </c>
@@ -4211,7 +4241,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A72" s="3" t="s">
         <v>350</v>
       </c>
@@ -4228,7 +4258,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A73" s="2" t="s">
         <v>352</v>
       </c>
@@ -4245,7 +4275,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A74" s="3" t="s">
         <v>354</v>
       </c>
@@ -4262,7 +4292,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A75" s="2" t="s">
         <v>356</v>
       </c>
@@ -4279,7 +4309,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A76" s="3" t="s">
         <v>358</v>
       </c>
@@ -4296,7 +4326,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A77" s="2" t="s">
         <v>360</v>
       </c>
@@ -4313,7 +4343,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A78" s="3" t="s">
         <v>362</v>
       </c>
@@ -4330,7 +4360,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A79" s="2" t="s">
         <v>364</v>
       </c>
@@ -4347,7 +4377,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A80" s="3" t="s">
         <v>366</v>
       </c>
@@ -4364,7 +4394,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A81" s="2" t="s">
         <v>368</v>
       </c>
@@ -4381,7 +4411,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A82" s="3" t="s">
         <v>370</v>
       </c>
@@ -4398,7 +4428,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A83" s="2" t="s">
         <v>372</v>
       </c>
@@ -4415,7 +4445,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A84" s="3" t="s">
         <v>374</v>
       </c>
@@ -4432,7 +4462,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A85" s="2" t="s">
         <v>376</v>
       </c>
@@ -4449,7 +4479,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A86" s="3" t="s">
         <v>378</v>
       </c>
@@ -4466,7 +4496,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A87" s="2" t="s">
         <v>380</v>
       </c>
@@ -4483,7 +4513,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A88" s="3" t="s">
         <v>382</v>
       </c>
@@ -4500,7 +4530,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A89" s="2" t="s">
         <v>384</v>
       </c>
@@ -4517,7 +4547,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A90" s="3" t="s">
         <v>386</v>
       </c>
@@ -4534,7 +4564,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A91" s="2" t="s">
         <v>388</v>
       </c>
@@ -4551,7 +4581,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A92" s="3" t="s">
         <v>390</v>
       </c>
@@ -4568,7 +4598,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A93" s="2" t="s">
         <v>392</v>
       </c>
@@ -4585,7 +4615,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A94" s="3" t="s">
         <v>394</v>
       </c>
@@ -4602,7 +4632,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A95" s="2" t="s">
         <v>396</v>
       </c>
@@ -4619,7 +4649,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A96" s="3" t="s">
         <v>398</v>
       </c>
@@ -4636,7 +4666,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A97" s="2" t="s">
         <v>400</v>
       </c>
@@ -4653,7 +4683,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A98" s="3" t="s">
         <v>402</v>
       </c>
@@ -4670,7 +4700,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A99" s="2" t="s">
         <v>404</v>
       </c>
@@ -4687,7 +4717,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A100" s="3" t="s">
         <v>406</v>
       </c>
@@ -4704,7 +4734,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A101" s="2" t="s">
         <v>408</v>
       </c>
@@ -4721,7 +4751,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A102" s="3" t="s">
         <v>410</v>
       </c>
@@ -4738,7 +4768,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A103" s="2" t="s">
         <v>412</v>
       </c>
@@ -4755,7 +4785,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A104" s="3" t="s">
         <v>414</v>
       </c>
@@ -4772,7 +4802,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A105" s="2" t="s">
         <v>416</v>
       </c>
@@ -4789,7 +4819,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A106" s="3" t="s">
         <v>418</v>
       </c>
@@ -4806,7 +4836,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A107" s="2" t="s">
         <v>420</v>
       </c>
@@ -4823,7 +4853,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A108" s="3" t="s">
         <v>422</v>
       </c>
@@ -4840,7 +4870,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A109" s="2" t="s">
         <v>424</v>
       </c>
@@ -4857,7 +4887,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A110" s="3" t="s">
         <v>426</v>
       </c>
@@ -4874,7 +4904,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A111" s="2" t="s">
         <v>428</v>
       </c>
@@ -4891,7 +4921,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A112" s="3" t="s">
         <v>430</v>
       </c>
@@ -4908,7 +4938,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A113" s="2" t="s">
         <v>432</v>
       </c>
@@ -4925,7 +4955,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A114" s="3" t="s">
         <v>434</v>
       </c>
@@ -4942,7 +4972,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A115" s="2" t="s">
         <v>436</v>
       </c>
@@ -4959,7 +4989,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A116" s="3" t="s">
         <v>438</v>
       </c>
@@ -4976,7 +5006,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A117" s="2" t="s">
         <v>440</v>
       </c>
@@ -4993,7 +5023,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A118" s="3" t="s">
         <v>442</v>
       </c>
@@ -5010,7 +5040,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A119" s="2" t="s">
         <v>444</v>
       </c>
@@ -5027,7 +5057,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A120" s="3" t="s">
         <v>446</v>
       </c>
@@ -5044,7 +5074,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A121" s="2" t="s">
         <v>448</v>
       </c>
@@ -5061,7 +5091,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A122" s="3" t="s">
         <v>450</v>
       </c>
@@ -5078,7 +5108,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A123" s="2" t="s">
         <v>452</v>
       </c>
@@ -5095,7 +5125,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A124" s="3" t="s">
         <v>454</v>
       </c>
@@ -5112,7 +5142,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A125" s="2" t="s">
         <v>456</v>
       </c>
@@ -5129,7 +5159,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A126" s="3" t="s">
         <v>458</v>
       </c>
@@ -5146,7 +5176,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A127" s="2" t="s">
         <v>460</v>
       </c>
@@ -5163,7 +5193,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A128" s="3" t="s">
         <v>462</v>
       </c>
@@ -5180,7 +5210,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A129" s="2" t="s">
         <v>464</v>
       </c>
@@ -5197,7 +5227,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A130" s="3" t="s">
         <v>466</v>
       </c>
@@ -5214,7 +5244,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A131" s="2" t="s">
         <v>468</v>
       </c>
@@ -5231,7 +5261,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A132" s="3" t="s">
         <v>470</v>
       </c>
@@ -5248,7 +5278,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A133" s="2" t="s">
         <v>472</v>
       </c>
@@ -5265,7 +5295,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A134" s="3" t="s">
         <v>474</v>
       </c>
@@ -5282,7 +5312,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A135" s="2" t="s">
         <v>476</v>
       </c>
@@ -5299,7 +5329,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A136" s="3" t="s">
         <v>478</v>
       </c>
@@ -5316,7 +5346,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A137" s="2" t="s">
         <v>480</v>
       </c>
@@ -5333,7 +5363,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A138" s="3" t="s">
         <v>482</v>
       </c>
@@ -5350,7 +5380,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A139" s="2" t="s">
         <v>484</v>
       </c>
@@ -5367,7 +5397,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A140" s="3" t="s">
         <v>486</v>
       </c>
@@ -5384,7 +5414,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A141" s="2" t="s">
         <v>488</v>
       </c>
@@ -5401,7 +5431,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A142" s="3" t="s">
         <v>490</v>
       </c>
@@ -5418,7 +5448,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A143" s="2" t="s">
         <v>492</v>
       </c>
@@ -5435,7 +5465,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A144" s="3" t="s">
         <v>494</v>
       </c>
@@ -5452,7 +5482,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A145" s="2" t="s">
         <v>496</v>
       </c>
@@ -5469,7 +5499,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A146" s="3" t="s">
         <v>498</v>
       </c>
@@ -5486,7 +5516,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A147" s="2" t="s">
         <v>501</v>
       </c>
@@ -5503,7 +5533,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A148" s="3" t="s">
         <v>503</v>
       </c>
@@ -5520,7 +5550,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A149" s="2" t="s">
         <v>505</v>
       </c>
@@ -5537,7 +5567,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A150" s="3" t="s">
         <v>507</v>
       </c>
@@ -5554,7 +5584,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A151" s="2" t="s">
         <v>509</v>
       </c>
@@ -5571,7 +5601,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A152" s="3" t="s">
         <v>511</v>
       </c>
@@ -5588,7 +5618,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A153" s="2" t="s">
         <v>513</v>
       </c>
@@ -5605,7 +5635,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A154" s="3" t="s">
         <v>515</v>
       </c>
@@ -5622,7 +5652,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A155" s="2" t="s">
         <v>517</v>
       </c>
@@ -5639,7 +5669,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A156" s="3" t="s">
         <v>519</v>
       </c>
@@ -5656,7 +5686,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A157" s="2" t="s">
         <v>521</v>
       </c>
@@ -5673,7 +5703,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A158" s="3" t="s">
         <v>523</v>
       </c>
@@ -5690,7 +5720,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A159" s="2" t="s">
         <v>525</v>
       </c>
@@ -5707,7 +5737,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A160" s="3" t="s">
         <v>527</v>
       </c>
@@ -5724,7 +5754,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A161" s="2" t="s">
         <v>529</v>
       </c>
@@ -5741,7 +5771,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A162" s="3" t="s">
         <v>531</v>
       </c>
@@ -5758,7 +5788,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A163" s="2" t="s">
         <v>533</v>
       </c>
@@ -5775,7 +5805,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A164" s="3" t="s">
         <v>535</v>
       </c>
@@ -5792,7 +5822,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A165" s="2" t="s">
         <v>537</v>
       </c>
@@ -5809,7 +5839,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A166" s="3" t="s">
         <v>539</v>
       </c>
@@ -5826,7 +5856,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A167" s="2" t="s">
         <v>541</v>
       </c>
@@ -5843,7 +5873,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A168" s="3" t="s">
         <v>543</v>
       </c>
@@ -5860,7 +5890,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A169" s="2" t="s">
         <v>545</v>
       </c>
@@ -5877,7 +5907,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A170" s="3" t="s">
         <v>547</v>
       </c>
@@ -5894,7 +5924,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A171" s="2" t="s">
         <v>549</v>
       </c>
@@ -5911,7 +5941,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A172" s="3" t="s">
         <v>551</v>
       </c>
@@ -5928,7 +5958,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A173" s="2" t="s">
         <v>553</v>
       </c>
@@ -5945,7 +5975,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A174" s="3" t="s">
         <v>555</v>
       </c>
@@ -5962,7 +5992,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A175" s="2" t="s">
         <v>557</v>
       </c>
@@ -5979,7 +6009,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A176" s="3" t="s">
         <v>559</v>
       </c>
@@ -5996,7 +6026,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A177" s="2" t="s">
         <v>561</v>
       </c>
@@ -6013,7 +6043,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A178" s="3" t="s">
         <v>563</v>
       </c>
@@ -6030,7 +6060,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A179" s="2" t="s">
         <v>565</v>
       </c>
@@ -6047,7 +6077,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A180" s="3" t="s">
         <v>567</v>
       </c>
@@ -6064,7 +6094,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A181" s="2" t="s">
         <v>569</v>
       </c>
@@ -6081,7 +6111,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A182" s="3" t="s">
         <v>571</v>
       </c>
@@ -6098,7 +6128,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A183" s="2" t="s">
         <v>573</v>
       </c>
@@ -6115,7 +6145,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A184" s="3" t="s">
         <v>575</v>
       </c>
@@ -6132,7 +6162,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A185" s="2" t="s">
         <v>577</v>
       </c>
@@ -6149,7 +6179,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A186" s="3" t="s">
         <v>579</v>
       </c>
@@ -6166,7 +6196,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A187" s="2" t="s">
         <v>581</v>
       </c>
@@ -6183,7 +6213,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A188" s="3" t="s">
         <v>583</v>
       </c>
@@ -6200,7 +6230,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A189" s="2" t="s">
         <v>585</v>
       </c>
@@ -6217,7 +6247,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A190" s="3" t="s">
         <v>587</v>
       </c>
@@ -6234,7 +6264,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A191" s="2" t="s">
         <v>589</v>
       </c>
@@ -6251,7 +6281,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A192" s="3" t="s">
         <v>591</v>
       </c>
@@ -6268,7 +6298,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A193" s="2" t="s">
         <v>593</v>
       </c>
@@ -6285,7 +6315,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A194" s="3" t="s">
         <v>595</v>
       </c>
@@ -6302,7 +6332,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A195" s="2" t="s">
         <v>597</v>
       </c>
@@ -6319,7 +6349,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A196" s="3" t="s">
         <v>599</v>
       </c>
@@ -6336,7 +6366,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A197" s="2" t="s">
         <v>601</v>
       </c>
@@ -6353,7 +6383,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A198" s="3" t="s">
         <v>603</v>
       </c>
@@ -6370,7 +6400,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A199" s="2" t="s">
         <v>605</v>
       </c>
@@ -6387,7 +6417,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A200" s="3" t="s">
         <v>607</v>
       </c>
@@ -6404,7 +6434,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A201" s="2" t="s">
         <v>609</v>
       </c>
@@ -6421,7 +6451,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A202" s="3" t="s">
         <v>611</v>
       </c>
@@ -6438,7 +6468,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A203" s="2" t="s">
         <v>613</v>
       </c>
@@ -6455,7 +6485,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A204" s="3" t="s">
         <v>615</v>
       </c>
@@ -6472,7 +6502,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A205" s="2" t="s">
         <v>617</v>
       </c>
@@ -6489,7 +6519,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A206" s="3" t="s">
         <v>619</v>
       </c>
@@ -6506,7 +6536,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A207" s="2" t="s">
         <v>621</v>
       </c>
@@ -6523,7 +6553,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A208" s="3" t="s">
         <v>623</v>
       </c>
@@ -6540,7 +6570,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A209" s="2" t="s">
         <v>625</v>
       </c>
@@ -6557,7 +6587,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A210" s="3" t="s">
         <v>627</v>
       </c>
@@ -6574,7 +6604,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A211" s="2" t="s">
         <v>629</v>
       </c>
@@ -6591,7 +6621,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A212" s="3" t="s">
         <v>631</v>
       </c>
@@ -6608,7 +6638,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A213" s="2" t="s">
         <v>633</v>
       </c>
@@ -6625,7 +6655,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A214" s="3" t="s">
         <v>635</v>
       </c>
@@ -6642,7 +6672,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A215" s="2" t="s">
         <v>637</v>
       </c>
@@ -6659,7 +6689,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A216" s="3" t="s">
         <v>639</v>
       </c>
@@ -6676,7 +6706,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A217" s="2" t="s">
         <v>641</v>
       </c>
@@ -6693,7 +6723,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A218" s="3" t="s">
         <v>643</v>
       </c>
@@ -6710,7 +6740,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A219" s="2" t="s">
         <v>645</v>
       </c>
@@ -6727,7 +6757,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A220" s="3" t="s">
         <v>647</v>
       </c>
@@ -6744,7 +6774,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A221" s="2" t="s">
         <v>649</v>
       </c>
@@ -6761,7 +6791,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A222" s="3" t="s">
         <v>651</v>
       </c>
@@ -6778,7 +6808,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A223" s="2" t="s">
         <v>653</v>
       </c>
@@ -6795,7 +6825,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A224" s="3" t="s">
         <v>655</v>
       </c>
@@ -6812,7 +6842,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A225" s="2" t="s">
         <v>657</v>
       </c>
@@ -6829,7 +6859,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A226" s="3" t="s">
         <v>659</v>
       </c>
@@ -6846,7 +6876,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A227" s="2" t="s">
         <v>661</v>
       </c>
@@ -6863,7 +6893,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A228" s="3" t="s">
         <v>663</v>
       </c>
@@ -6880,7 +6910,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A229" s="2" t="s">
         <v>665</v>
       </c>
@@ -6897,7 +6927,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A230" s="3" t="s">
         <v>667</v>
       </c>
@@ -6914,7 +6944,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A231" s="2" t="s">
         <v>669</v>
       </c>
@@ -6931,7 +6961,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A232" s="3" t="s">
         <v>671</v>
       </c>
@@ -6948,7 +6978,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A233" s="2" t="s">
         <v>673</v>
       </c>
@@ -6965,7 +6995,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A234" s="3" t="s">
         <v>675</v>
       </c>
@@ -6982,7 +7012,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A235" s="2" t="s">
         <v>677</v>
       </c>
@@ -6999,7 +7029,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A236" s="3" t="s">
         <v>688</v>
       </c>
@@ -7016,7 +7046,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A237" s="2" t="s">
         <v>690</v>
       </c>
@@ -7033,7 +7063,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A238" s="3" t="s">
         <v>692</v>
       </c>
@@ -7050,7 +7080,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A239" s="2" t="s">
         <v>694</v>
       </c>
@@ -7067,7 +7097,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A240" s="3" t="s">
         <v>696</v>
       </c>
@@ -7084,7 +7114,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A241" s="2" t="s">
         <v>698</v>
       </c>
@@ -7101,7 +7131,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A242" s="3" t="s">
         <v>700</v>
       </c>
@@ -7118,7 +7148,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A243" s="2" t="s">
         <v>702</v>
       </c>
@@ -7135,7 +7165,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A244" s="3" t="s">
         <v>704</v>
       </c>
@@ -7152,7 +7182,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A245" s="2" t="s">
         <v>706</v>
       </c>
@@ -7169,7 +7199,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A246" s="3" t="s">
         <v>708</v>
       </c>
@@ -7186,7 +7216,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A247" s="2" t="s">
         <v>710</v>
       </c>
@@ -7203,7 +7233,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A248" s="3" t="s">
         <v>712</v>
       </c>
@@ -7220,7 +7250,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A249" s="2" t="s">
         <v>714</v>
       </c>
@@ -7237,7 +7267,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A250" s="3" t="s">
         <v>716</v>
       </c>
@@ -7254,7 +7284,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A251" s="2" t="s">
         <v>718</v>
       </c>
@@ -7271,7 +7301,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A252" s="2" t="s">
         <v>257</v>
       </c>
@@ -7288,7 +7318,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A253" s="3" t="s">
         <v>720</v>
       </c>
@@ -7305,7 +7335,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A254" s="2" t="s">
         <v>722</v>
       </c>
@@ -7322,7 +7352,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A255" s="3" t="s">
         <v>724</v>
       </c>
@@ -7339,7 +7369,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A256" s="2" t="s">
         <v>726</v>
       </c>
@@ -7356,7 +7386,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A257" s="3" t="s">
         <v>728</v>
       </c>
@@ -7373,7 +7403,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A258" s="2" t="s">
         <v>730</v>
       </c>
@@ -7390,7 +7420,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A259" s="3" t="s">
         <v>259</v>
       </c>
@@ -7407,7 +7437,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A260" s="3" t="s">
         <v>732</v>
       </c>
@@ -7424,7 +7454,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A261" s="2" t="s">
         <v>734</v>
       </c>
@@ -7441,7 +7471,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A262" s="3" t="s">
         <v>736</v>
       </c>
@@ -7458,7 +7488,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A263" s="2" t="s">
         <v>738</v>
       </c>
@@ -7475,7 +7505,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A264" s="3" t="s">
         <v>740</v>
       </c>
@@ -7492,7 +7522,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A265" s="2" t="s">
         <v>742</v>
       </c>
@@ -7509,7 +7539,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A266" s="3" t="s">
         <v>744</v>
       </c>
@@ -7526,7 +7556,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A267" s="2" t="s">
         <v>746</v>
       </c>
@@ -7543,7 +7573,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A268" s="3" t="s">
         <v>748</v>
       </c>
@@ -7560,7 +7590,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A269" s="2" t="s">
         <v>750</v>
       </c>
@@ -7577,7 +7607,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A270" s="3" t="s">
         <v>752</v>
       </c>
@@ -7594,7 +7624,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A271" s="2" t="s">
         <v>754</v>
       </c>
@@ -7611,7 +7641,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A272" s="3" t="s">
         <v>756</v>
       </c>
@@ -7628,7 +7658,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A273" s="2" t="s">
         <v>758</v>
       </c>
@@ -7645,7 +7675,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A274" s="3" t="s">
         <v>760</v>
       </c>
@@ -7662,7 +7692,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A275" s="2" t="s">
         <v>762</v>
       </c>
@@ -7679,7 +7709,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A276" s="2" t="s">
         <v>5</v>
       </c>
@@ -7696,7 +7726,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A277" s="3" t="s">
         <v>764</v>
       </c>
@@ -7713,7 +7743,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A278" s="2" t="s">
         <v>766</v>
       </c>
@@ -7730,7 +7760,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="279" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A279" s="3" t="s">
         <v>768</v>
       </c>
@@ -7747,7 +7777,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="280" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A280" s="2" t="s">
         <v>770</v>
       </c>
@@ -7764,7 +7794,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="281" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A281" s="3" t="s">
         <v>772</v>
       </c>
@@ -7781,7 +7811,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="282" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A282" s="2" t="s">
         <v>774</v>
       </c>
@@ -7798,7 +7828,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="283" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A283" s="3" t="s">
         <v>776</v>
       </c>
@@ -7815,7 +7845,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="284" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A284" s="2" t="s">
         <v>778</v>
       </c>
@@ -7832,7 +7862,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="285" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A285" s="3" t="s">
         <v>780</v>
       </c>
@@ -7849,7 +7879,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="286" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A286" s="2" t="s">
         <v>782</v>
       </c>
@@ -7866,7 +7896,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="287" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A287" s="3" t="s">
         <v>784</v>
       </c>
@@ -7883,7 +7913,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="288" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A288" s="2" t="s">
         <v>786</v>
       </c>
@@ -7900,7 +7930,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A289" s="3" t="s">
         <v>788</v>
       </c>
@@ -7917,7 +7947,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A290" s="2" t="s">
         <v>790</v>
       </c>
@@ -7934,7 +7964,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A291" s="3" t="s">
         <v>792</v>
       </c>
@@ -7951,7 +7981,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A292" s="2" t="s">
         <v>794</v>
       </c>
@@ -7968,7 +7998,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A293" s="3" t="s">
         <v>796</v>
       </c>
@@ -7985,7 +8015,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A294" s="2" t="s">
         <v>798</v>
       </c>
@@ -8002,7 +8032,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A295" s="3" t="s">
         <v>800</v>
       </c>
@@ -8019,7 +8049,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A296" s="2" t="s">
         <v>802</v>
       </c>
@@ -8036,7 +8066,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A297" s="3" t="s">
         <v>804</v>
       </c>
@@ -8053,7 +8083,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A298" s="2" t="s">
         <v>806</v>
       </c>
@@ -8070,7 +8100,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A299" s="3" t="s">
         <v>808</v>
       </c>
@@ -8087,7 +8117,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A300" s="2" t="s">
         <v>810</v>
       </c>
@@ -8104,7 +8134,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="301" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A301" s="3" t="s">
         <v>812</v>
       </c>
@@ -8121,7 +8151,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A302" s="2" t="s">
         <v>814</v>
       </c>
@@ -8138,7 +8168,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A303" s="3" t="s">
         <v>816</v>
       </c>
@@ -8155,7 +8185,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="304" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A304" s="2" t="s">
         <v>818</v>
       </c>
@@ -8172,7 +8202,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="305" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A305" s="3" t="s">
         <v>820</v>
       </c>
@@ -8189,7 +8219,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="306" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A306" s="3" t="s">
         <v>10</v>
       </c>
@@ -8206,7 +8236,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="307" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A307" s="2" t="s">
         <v>12</v>
       </c>
@@ -8223,7 +8253,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="308" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A308" s="2" t="s">
         <v>822</v>
       </c>
@@ -8240,7 +8270,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="309" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A309" s="3" t="s">
         <v>824</v>
       </c>
@@ -8257,7 +8287,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="310" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A310" s="2" t="s">
         <v>826</v>
       </c>
@@ -8274,7 +8304,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="311" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A311" s="3" t="s">
         <v>828</v>
       </c>
@@ -8291,7 +8321,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="312" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A312" s="2" t="s">
         <v>830</v>
       </c>
@@ -8308,7 +8338,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="313" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A313" s="3" t="s">
         <v>832</v>
       </c>
@@ -8325,7 +8355,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="314" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A314" s="2" t="s">
         <v>834</v>
       </c>
@@ -8342,7 +8372,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="315" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A315" s="3" t="s">
         <v>836</v>
       </c>
@@ -8359,7 +8389,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="316" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A316" s="2" t="s">
         <v>838</v>
       </c>
@@ -8376,7 +8406,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="317" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A317" s="3" t="s">
         <v>840</v>
       </c>
@@ -8393,7 +8423,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="318" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A318" s="2" t="s">
         <v>842</v>
       </c>
@@ -8410,7 +8440,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="319" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A319" s="3" t="s">
         <v>844</v>
       </c>
@@ -8427,7 +8457,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="320" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A320" s="2" t="s">
         <v>846</v>
       </c>
@@ -8444,7 +8474,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="321" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A321" s="3" t="s">
         <v>848</v>
       </c>
@@ -8461,7 +8491,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="322" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A322" s="2" t="s">
         <v>850</v>
       </c>
@@ -8478,7 +8508,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="323" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A323" s="3" t="s">
         <v>852</v>
       </c>
@@ -8495,7 +8525,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="324" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A324" s="2" t="s">
         <v>261</v>
       </c>
@@ -8512,7 +8542,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="325" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A325" s="3" t="s">
         <v>14</v>
       </c>
@@ -8529,7 +8559,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="326" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A326" s="2" t="s">
         <v>16</v>
       </c>
@@ -8546,7 +8576,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="327" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A327" s="3" t="s">
         <v>18</v>
       </c>
@@ -8563,7 +8593,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="328" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A328" s="2" t="s">
         <v>20</v>
       </c>
@@ -8580,7 +8610,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="329" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A329" s="3" t="s">
         <v>263</v>
       </c>
@@ -8597,7 +8627,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="330" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A330" s="2" t="s">
         <v>265</v>
       </c>
@@ -8614,7 +8644,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="331" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A331" s="3" t="s">
         <v>22</v>
       </c>
@@ -8631,7 +8661,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="332" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A332" s="2" t="s">
         <v>24</v>
       </c>
@@ -8648,7 +8678,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="333" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A333" s="3" t="s">
         <v>26</v>
       </c>
@@ -8665,7 +8695,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="334" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A334" s="2" t="s">
         <v>28</v>
       </c>
@@ -8682,7 +8712,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="335" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A335" s="3" t="s">
         <v>30</v>
       </c>
@@ -8699,7 +8729,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="336" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A336" s="3" t="s">
         <v>267</v>
       </c>
@@ -8716,7 +8746,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="337" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A337" s="2" t="s">
         <v>32</v>
       </c>
@@ -8733,7 +8763,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="338" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A338" s="2" t="s">
         <v>269</v>
       </c>
@@ -8750,7 +8780,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="339" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A339" s="2" t="s">
         <v>854</v>
       </c>
@@ -8767,7 +8797,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="340" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A340" s="3" t="s">
         <v>856</v>
       </c>
@@ -8784,7 +8814,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="341" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A341" s="3" t="s">
         <v>34</v>
       </c>
@@ -8801,7 +8831,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="342" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A342" s="2" t="s">
         <v>36</v>
       </c>
@@ -8818,7 +8848,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="343" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A343" s="3" t="s">
         <v>38</v>
       </c>
@@ -8835,7 +8865,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="344" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A344" s="2" t="s">
         <v>40</v>
       </c>
@@ -8852,7 +8882,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="345" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A345" s="3" t="s">
         <v>42</v>
       </c>
@@ -8869,7 +8899,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="346" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A346" s="2" t="s">
         <v>44</v>
       </c>
@@ -8886,7 +8916,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="347" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A347" s="3" t="s">
         <v>46</v>
       </c>
@@ -8903,7 +8933,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="348" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A348" s="2" t="s">
         <v>48</v>
       </c>
@@ -8920,7 +8950,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="349" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A349" s="3" t="s">
         <v>50</v>
       </c>
@@ -8937,7 +8967,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="350" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A350" s="2" t="s">
         <v>52</v>
       </c>
@@ -8954,7 +8984,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="351" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A351" s="3" t="s">
         <v>54</v>
       </c>
@@ -8971,7 +9001,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="352" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A352" s="2" t="s">
         <v>56</v>
       </c>
@@ -8988,7 +9018,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="353" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A353" s="3" t="s">
         <v>58</v>
       </c>
@@ -9005,7 +9035,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="354" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A354" s="3" t="s">
         <v>271</v>
       </c>
@@ -9022,7 +9052,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="355" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A355" s="2" t="s">
         <v>273</v>
       </c>
@@ -9039,7 +9069,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="356" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A356" s="2" t="s">
         <v>858</v>
       </c>
@@ -9056,7 +9086,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="357" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A357" s="2" t="s">
         <v>60</v>
       </c>
@@ -9073,7 +9103,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="358" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A358" s="3" t="s">
         <v>62</v>
       </c>
@@ -9090,7 +9120,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="359" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A359" s="2" t="s">
         <v>64</v>
       </c>
@@ -9107,7 +9137,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="360" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A360" s="3" t="s">
         <v>275</v>
       </c>
@@ -9124,7 +9154,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="361" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A361" s="3" t="s">
         <v>66</v>
       </c>
@@ -9141,7 +9171,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="362" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A362" s="2" t="s">
         <v>68</v>
       </c>
@@ -9158,7 +9188,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="363" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A363" s="3" t="s">
         <v>70</v>
       </c>
@@ -9175,7 +9205,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="364" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A364" s="2" t="s">
         <v>72</v>
       </c>
@@ -9192,7 +9222,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="365" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A365" s="2" t="s">
         <v>277</v>
       </c>
@@ -9209,7 +9239,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="366" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A366" s="3" t="s">
         <v>74</v>
       </c>
@@ -9226,7 +9256,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="367" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A367" s="2" t="s">
         <v>76</v>
       </c>
@@ -9243,7 +9273,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="368" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A368" s="3" t="s">
         <v>860</v>
       </c>
@@ -9260,7 +9290,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="369" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A369" s="3" t="s">
         <v>78</v>
       </c>
@@ -9277,7 +9307,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="370" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A370" s="2" t="s">
         <v>80</v>
       </c>
@@ -9294,7 +9324,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="371" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A371" s="3" t="s">
         <v>82</v>
       </c>
@@ -9311,7 +9341,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="372" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A372" s="2" t="s">
         <v>84</v>
       </c>
@@ -9328,7 +9358,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="373" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A373" s="3" t="s">
         <v>86</v>
       </c>
@@ -9345,7 +9375,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="374" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A374" s="2" t="s">
         <v>88</v>
       </c>
@@ -9362,7 +9392,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="375" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A375" s="3" t="s">
         <v>279</v>
       </c>
@@ -9379,7 +9409,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="376" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A376" s="3" t="s">
         <v>90</v>
       </c>
@@ -9396,7 +9426,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="377" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A377" s="2" t="s">
         <v>92</v>
       </c>
@@ -9413,7 +9443,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="378" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A378" s="2" t="s">
         <v>281</v>
       </c>
@@ -9430,7 +9460,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="379" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A379" s="3" t="s">
         <v>94</v>
       </c>
@@ -9447,7 +9477,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="380" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A380" s="2" t="s">
         <v>96</v>
       </c>
@@ -9464,7 +9494,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="381" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A381" s="3" t="s">
         <v>283</v>
       </c>
@@ -9481,7 +9511,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="382" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A382" s="3" t="s">
         <v>98</v>
       </c>
@@ -9498,7 +9528,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="383" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="383" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A383" s="2" t="s">
         <v>100</v>
       </c>
@@ -9515,7 +9545,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="384" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="384" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A384" s="3" t="s">
         <v>102</v>
       </c>
@@ -9532,7 +9562,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="385" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="385" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A385" s="2" t="s">
         <v>104</v>
       </c>
@@ -9549,7 +9579,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="386" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="386" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A386" s="2" t="s">
         <v>285</v>
       </c>
@@ -9566,7 +9596,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="387" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="387" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A387" s="3" t="s">
         <v>106</v>
       </c>
@@ -9583,7 +9613,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="388" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="388" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A388" s="2" t="s">
         <v>108</v>
       </c>
@@ -9600,7 +9630,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="389" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="389" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A389" s="3" t="s">
         <v>110</v>
       </c>
@@ -9617,7 +9647,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="390" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="390" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A390" s="2" t="s">
         <v>112</v>
       </c>
@@ -9634,7 +9664,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="391" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="391" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A391" s="3" t="s">
         <v>114</v>
       </c>
@@ -9651,7 +9681,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="392" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="392" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A392" s="2" t="s">
         <v>116</v>
       </c>
@@ -9668,7 +9698,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="393" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="393" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A393" s="3" t="s">
         <v>118</v>
       </c>
@@ -9685,7 +9715,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="394" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="394" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A394" s="2" t="s">
         <v>120</v>
       </c>
@@ -9702,7 +9732,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="395" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="395" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A395" s="3" t="s">
         <v>122</v>
       </c>
@@ -9719,7 +9749,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="396" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="396" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A396" s="3" t="s">
         <v>287</v>
       </c>
@@ -9736,7 +9766,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="397" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="397" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A397" s="2" t="s">
         <v>124</v>
       </c>
@@ -9753,7 +9783,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="398" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="398" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A398" s="3" t="s">
         <v>126</v>
       </c>
@@ -9770,7 +9800,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="399" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="399" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A399" s="2" t="s">
         <v>128</v>
       </c>
@@ -9787,7 +9817,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="400" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="400" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A400" s="3" t="s">
         <v>130</v>
       </c>
@@ -9804,7 +9834,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="401" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="401" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A401" s="2" t="s">
         <v>289</v>
       </c>
@@ -9821,7 +9851,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="402" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="402" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A402" s="2" t="s">
         <v>132</v>
       </c>
@@ -9838,7 +9868,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="403" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="403" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A403" s="3" t="s">
         <v>134</v>
       </c>
@@ -9855,7 +9885,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="404" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="404" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A404" s="2" t="s">
         <v>136</v>
       </c>
@@ -9872,7 +9902,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="405" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="405" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A405" s="3" t="s">
         <v>138</v>
       </c>
@@ -9889,7 +9919,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="406" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="406" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A406" s="3" t="s">
         <v>291</v>
       </c>
@@ -9906,7 +9936,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="407" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="407" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A407" s="2" t="s">
         <v>293</v>
       </c>
@@ -9923,7 +9953,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="408" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="408" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A408" s="3" t="s">
         <v>295</v>
       </c>
@@ -9940,7 +9970,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="409" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="409" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A409" s="2" t="s">
         <v>297</v>
       </c>
@@ -9957,7 +9987,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="410" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="410" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A410" s="2" t="s">
         <v>140</v>
       </c>
@@ -9974,7 +10004,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="411" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="411" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A411" s="3" t="s">
         <v>142</v>
       </c>
@@ -9991,7 +10021,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="412" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="412" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A412" s="2" t="s">
         <v>144</v>
       </c>
@@ -10008,7 +10038,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="413" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="413" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A413" s="3" t="s">
         <v>299</v>
       </c>
@@ -10025,7 +10055,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="414" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="414" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A414" s="3" t="s">
         <v>146</v>
       </c>
@@ -10042,7 +10072,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="415" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="415" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A415" s="2" t="s">
         <v>148</v>
       </c>
@@ -10059,7 +10089,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="416" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="416" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A416" s="3" t="s">
         <v>150</v>
       </c>
@@ -10076,7 +10106,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="417" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="417" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A417" s="2" t="s">
         <v>301</v>
       </c>
@@ -10093,7 +10123,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="418" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="418" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A418" s="3" t="s">
         <v>303</v>
       </c>
@@ -10110,7 +10140,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="419" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="419" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A419" s="2" t="s">
         <v>152</v>
       </c>
@@ -10127,7 +10157,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="420" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="420" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A420" s="3" t="s">
         <v>154</v>
       </c>
@@ -10144,7 +10174,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="421" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="421" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A421" s="2" t="s">
         <v>156</v>
       </c>
@@ -10161,7 +10191,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="422" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="422" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A422" s="3" t="s">
         <v>158</v>
       </c>
@@ -10178,7 +10208,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="423" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="423" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A423" s="2" t="s">
         <v>305</v>
       </c>
@@ -10195,7 +10225,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="424" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="424" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A424" s="3" t="s">
         <v>307</v>
       </c>
@@ -10212,7 +10242,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="425" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="425" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A425" s="2" t="s">
         <v>309</v>
       </c>
@@ -10229,7 +10259,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="426" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="426" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A426" s="3" t="s">
         <v>311</v>
       </c>
@@ -10246,7 +10276,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="427" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="427" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A427" s="2" t="s">
         <v>313</v>
       </c>
@@ -10260,6 +10290,159 @@
         <v>162</v>
       </c>
       <c r="E427" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="430" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A430" s="2">
+        <v>210303</v>
+      </c>
+      <c r="B430" s="2" t="s">
+        <v>864</v>
+      </c>
+      <c r="C430" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D430" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="E430" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="431" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A431" s="3">
+        <v>211560</v>
+      </c>
+      <c r="B431" s="3" t="s">
+        <v>865</v>
+      </c>
+      <c r="C431" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D431" s="3" t="s">
+        <v>681</v>
+      </c>
+      <c r="E431" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="432" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A432" s="2">
+        <v>211701</v>
+      </c>
+      <c r="B432" s="2" t="s">
+        <v>866</v>
+      </c>
+      <c r="C432" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D432" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="E432" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="433" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A433" s="2">
+        <v>211892</v>
+      </c>
+      <c r="B433" s="2" t="s">
+        <v>867</v>
+      </c>
+      <c r="C433" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D433" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="E433" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="434" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A434" s="3">
+        <v>200502</v>
+      </c>
+      <c r="B434" s="3" t="s">
+        <v>868</v>
+      </c>
+      <c r="C434" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D434" s="3" t="s">
+        <v>681</v>
+      </c>
+      <c r="E434" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="435" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A435" s="2">
+        <v>200764</v>
+      </c>
+      <c r="B435" s="2" t="s">
+        <v>869</v>
+      </c>
+      <c r="C435" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D435" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="E435" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="436" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A436" s="2">
+        <v>201076</v>
+      </c>
+      <c r="B436" s="2" t="s">
+        <v>870</v>
+      </c>
+      <c r="C436" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D436" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="E436" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="437" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A437" s="3">
+        <v>201249</v>
+      </c>
+      <c r="B437" s="3" t="s">
+        <v>871</v>
+      </c>
+      <c r="C437" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D437" s="3" t="s">
+        <v>681</v>
+      </c>
+      <c r="E437" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="438" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A438" s="2">
+        <v>201538</v>
+      </c>
+      <c r="B438" s="2" t="s">
+        <v>872</v>
+      </c>
+      <c r="C438" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D438" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="E438" s="2" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>